<commit_message>
Update Analysis Add-ins Excel file
Replaced 1_Analysis_Add-ins.xlsx with a new version. The update may include revised data, formulas, or add-in references to support advanced data analytics tasks.
</commit_message>
<xml_diff>
--- a/6_Advanced_Data_Analytics/1_Analysis_Add-ins.xlsx
+++ b/6_Advanced_Data_Analytics/1_Analysis_Add-ins.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\OneDrive\Desktop\Projects\Excel_For_Data_Analytics_1\Excel_Project_Data_Analytics\6_Advanced_Data_Analytics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05450743-BD6B-47C4-91B5-9F11F177E9A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{058942E5-9F31-43EB-8D25-CA2FA8880EB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="4" activeTab="7" xr2:uid="{6C37AC85-509F-4D10-9DB1-F70D16D6FBAB}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{6C37AC85-509F-4D10-9DB1-F70D16D6FBAB}"/>
   </bookViews>
   <sheets>
     <sheet name="Forecast_Original" sheetId="7" r:id="rId1"/>

</xml_diff>